<commit_message>
MP adding the wrong column
</commit_message>
<xml_diff>
--- a/howell4.xlsx
+++ b/howell4.xlsx
@@ -506,7 +506,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>For public domain. No rights reserved. Generated on Apr 08, 2026.</t>
+          <t>For public domain. No rights reserved. Generated on Apr 22, 2026.</t>
         </is>
       </c>
     </row>
@@ -590,12 +590,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Name 53</t>
+          <t>Name 52</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Name 61</t>
+          <t>Name 86</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -613,12 +613,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Name 79</t>
+          <t>Name 66</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Name 89</t>
+          <t>Name 50</t>
         </is>
       </c>
       <c r="D11" s="4">
@@ -636,12 +636,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Name 49</t>
+          <t>Name 24</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Name 59</t>
+          <t>Name 12</t>
         </is>
       </c>
       <c r="D12" s="4">
@@ -659,12 +659,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Name 42</t>
+          <t>Name 54</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Name 74</t>
+          <t>Name 71</t>
         </is>
       </c>
       <c r="D13" s="4">

</xml_diff>

<commit_message>
average as 0.5, not empty string
</commit_message>
<xml_diff>
--- a/howell4.xlsx
+++ b/howell4.xlsx
@@ -506,7 +506,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>For public domain. No rights reserved. Generated on Apr 22, 2026.</t>
+          <t>For public domain. No rights reserved. Generated on Apr 23, 2026.</t>
         </is>
       </c>
     </row>
@@ -590,12 +590,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Name 75</t>
+          <t>Name 12</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Name 65</t>
+          <t>Name 64</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -613,12 +613,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Name 39</t>
+          <t>Name 83</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Name 68</t>
+          <t>Name 20</t>
         </is>
       </c>
       <c r="D11" s="4">
@@ -636,12 +636,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Name 16</t>
+          <t>Name 81</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Name 42</t>
+          <t>Name 45</t>
         </is>
       </c>
       <c r="D12" s="4">
@@ -659,12 +659,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>Name 54</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>Name 14</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Name 20</t>
         </is>
       </c>
       <c r="D13" s="4">
@@ -957,11 +957,11 @@
         <v/>
       </c>
       <c r="U3" s="14">
-        <f>IF(ISNUMBER(S3),IF(ISNUMBER(S4),IF(S3&gt;S4,1.0,IF(S3=S4,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S3),IF(ISNUMBER(S4),IF(S3&gt;S4,1.0,IF(S3=S4,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V3">
-        <f>IF(ISNUMBER(T3),IF(ISNUMBER(T4),IF(T3&gt;T4,1.0,IF(T3=T4,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T3),IF(ISNUMBER(T4),IF(T3&gt;T4,1.0,IF(T3=T4,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W3" s="14">
@@ -1052,11 +1052,11 @@
         <v/>
       </c>
       <c r="U4" s="21">
-        <f>IF(ISNUMBER(S4),IF(ISNUMBER(S3),IF(S4&gt;S3,1.0,IF(S4=S3,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S4),IF(ISNUMBER(S3),IF(S4&gt;S3,1.0,IF(S4=S3,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V4" s="15">
-        <f>IF(ISNUMBER(T4),IF(ISNUMBER(T3),IF(T4&gt;T3,1.0,IF(T4=T3,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T4),IF(ISNUMBER(T3),IF(T4&gt;T3,1.0,IF(T4=T3,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W4" s="21">
@@ -1149,11 +1149,11 @@
         <v/>
       </c>
       <c r="U5" s="14">
-        <f>IF(ISNUMBER(S5),IF(ISNUMBER(S6),IF(S5&gt;S6,1.0,IF(S5=S6,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S5),IF(ISNUMBER(S6),IF(S5&gt;S6,1.0,IF(S5=S6,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V5">
-        <f>IF(ISNUMBER(T5),IF(ISNUMBER(T6),IF(T5&gt;T6,1.0,IF(T5=T6,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T5),IF(ISNUMBER(T6),IF(T5&gt;T6,1.0,IF(T5=T6,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W5" s="14">
@@ -1244,11 +1244,11 @@
         <v/>
       </c>
       <c r="U6" s="21">
-        <f>IF(ISNUMBER(S6),IF(ISNUMBER(S5),IF(S6&gt;S5,1.0,IF(S6=S5,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S6),IF(ISNUMBER(S5),IF(S6&gt;S5,1.0,IF(S6=S5,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V6" s="15">
-        <f>IF(ISNUMBER(T6),IF(ISNUMBER(T5),IF(T6&gt;T5,1.0,IF(T6=T5,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T6),IF(ISNUMBER(T5),IF(T6&gt;T5,1.0,IF(T6=T5,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W6" s="21">
@@ -1341,11 +1341,11 @@
         <v/>
       </c>
       <c r="U7" s="14">
-        <f>IF(ISNUMBER(S7),IF(ISNUMBER(S8),IF(S7&gt;S8,1.0,IF(S7=S8,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S7),IF(ISNUMBER(S8),IF(S7&gt;S8,1.0,IF(S7=S8,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V7">
-        <f>IF(ISNUMBER(T7),IF(ISNUMBER(T8),IF(T7&gt;T8,1.0,IF(T7=T8,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T7),IF(ISNUMBER(T8),IF(T7&gt;T8,1.0,IF(T7=T8,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W7" s="14">
@@ -1436,11 +1436,11 @@
         <v/>
       </c>
       <c r="U8" s="21">
-        <f>IF(ISNUMBER(S8),IF(ISNUMBER(S7),IF(S8&gt;S7,1.0,IF(S8=S7,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S8),IF(ISNUMBER(S7),IF(S8&gt;S7,1.0,IF(S8=S7,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V8" s="15">
-        <f>IF(ISNUMBER(T8),IF(ISNUMBER(T7),IF(T8&gt;T7,1.0,IF(T8=T7,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T8),IF(ISNUMBER(T7),IF(T8&gt;T7,1.0,IF(T8=T7,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W8" s="21">
@@ -1533,11 +1533,11 @@
         <v/>
       </c>
       <c r="U9" s="14">
-        <f>IF(ISNUMBER(S9),IF(ISNUMBER(S10),IF(S9&gt;S10,1.0,IF(S9=S10,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S9),IF(ISNUMBER(S10),IF(S9&gt;S10,1.0,IF(S9=S10,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V9">
-        <f>IF(ISNUMBER(T9),IF(ISNUMBER(T10),IF(T9&gt;T10,1.0,IF(T9=T10,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T9),IF(ISNUMBER(T10),IF(T9&gt;T10,1.0,IF(T9=T10,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W9" s="14">
@@ -1628,11 +1628,11 @@
         <v/>
       </c>
       <c r="U10" s="21">
-        <f>IF(ISNUMBER(S10),IF(ISNUMBER(S9),IF(S10&gt;S9,1.0,IF(S10=S9,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S10),IF(ISNUMBER(S9),IF(S10&gt;S9,1.0,IF(S10=S9,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V10" s="15">
-        <f>IF(ISNUMBER(T10),IF(ISNUMBER(T9),IF(T10&gt;T9,1.0,IF(T10=T9,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T10),IF(ISNUMBER(T9),IF(T10&gt;T9,1.0,IF(T10=T9,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W10" s="21">
@@ -1725,11 +1725,11 @@
         <v/>
       </c>
       <c r="U11" s="14">
-        <f>IF(ISNUMBER(S11),IF(ISNUMBER(S12),IF(S11&gt;S12,1.0,IF(S11=S12,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S11),IF(ISNUMBER(S12),IF(S11&gt;S12,1.0,IF(S11=S12,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V11">
-        <f>IF(ISNUMBER(T11),IF(ISNUMBER(T12),IF(T11&gt;T12,1.0,IF(T11=T12,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T11),IF(ISNUMBER(T12),IF(T11&gt;T12,1.0,IF(T11=T12,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W11" s="14">
@@ -1820,11 +1820,11 @@
         <v/>
       </c>
       <c r="U12" s="21">
-        <f>IF(ISNUMBER(S12),IF(ISNUMBER(S11),IF(S12&gt;S11,1.0,IF(S12=S11,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S12),IF(ISNUMBER(S11),IF(S12&gt;S11,1.0,IF(S12=S11,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V12" s="15">
-        <f>IF(ISNUMBER(T12),IF(ISNUMBER(T11),IF(T12&gt;T11,1.0,IF(T12=T11,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T12),IF(ISNUMBER(T11),IF(T12&gt;T11,1.0,IF(T12=T11,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W12" s="21">
@@ -1917,11 +1917,11 @@
         <v/>
       </c>
       <c r="U13" s="14">
-        <f>IF(ISNUMBER(S13),IF(ISNUMBER(S14),IF(S13&gt;S14,1.0,IF(S13=S14,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S13),IF(ISNUMBER(S14),IF(S13&gt;S14,1.0,IF(S13=S14,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V13">
-        <f>IF(ISNUMBER(T13),IF(ISNUMBER(T14),IF(T13&gt;T14,1.0,IF(T13=T14,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T13),IF(ISNUMBER(T14),IF(T13&gt;T14,1.0,IF(T13=T14,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W13" s="14">
@@ -2012,11 +2012,11 @@
         <v/>
       </c>
       <c r="U14" s="21">
-        <f>IF(ISNUMBER(S14),IF(ISNUMBER(S13),IF(S14&gt;S13,1.0,IF(S14=S13,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S14),IF(ISNUMBER(S13),IF(S14&gt;S13,1.0,IF(S14=S13,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V14" s="15">
-        <f>IF(ISNUMBER(T14),IF(ISNUMBER(T13),IF(T14&gt;T13,1.0,IF(T14=T13,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T14),IF(ISNUMBER(T13),IF(T14&gt;T13,1.0,IF(T14=T13,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W14" s="21">
@@ -2109,11 +2109,11 @@
         <v/>
       </c>
       <c r="U15" s="14">
-        <f>IF(ISNUMBER(S15),IF(ISNUMBER(S16),IF(S15&gt;S16,1.0,IF(S15=S16,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S15),IF(ISNUMBER(S16),IF(S15&gt;S16,1.0,IF(S15=S16,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V15">
-        <f>IF(ISNUMBER(T15),IF(ISNUMBER(T16),IF(T15&gt;T16,1.0,IF(T15=T16,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T15),IF(ISNUMBER(T16),IF(T15&gt;T16,1.0,IF(T15=T16,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W15" s="14">
@@ -2204,11 +2204,11 @@
         <v/>
       </c>
       <c r="U16" s="21">
-        <f>IF(ISNUMBER(S16),IF(ISNUMBER(S15),IF(S16&gt;S15,1.0,IF(S16=S15,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S16),IF(ISNUMBER(S15),IF(S16&gt;S15,1.0,IF(S16=S15,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V16" s="15">
-        <f>IF(ISNUMBER(T16),IF(ISNUMBER(T15),IF(T16&gt;T15,1.0,IF(T16=T15,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T16),IF(ISNUMBER(T15),IF(T16&gt;T15,1.0,IF(T16=T15,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W16" s="21">
@@ -2301,11 +2301,11 @@
         <v/>
       </c>
       <c r="U17" s="14">
-        <f>IF(ISNUMBER(S17),IF(ISNUMBER(S18),IF(S17&gt;S18,1.0,IF(S17=S18,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S17),IF(ISNUMBER(S18),IF(S17&gt;S18,1.0,IF(S17=S18,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V17">
-        <f>IF(ISNUMBER(T17),IF(ISNUMBER(T18),IF(T17&gt;T18,1.0,IF(T17=T18,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T17),IF(ISNUMBER(T18),IF(T17&gt;T18,1.0,IF(T17=T18,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W17" s="14">
@@ -2396,11 +2396,11 @@
         <v/>
       </c>
       <c r="U18" s="21">
-        <f>IF(ISNUMBER(S18),IF(ISNUMBER(S17),IF(S18&gt;S17,1.0,IF(S18=S17,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S18),IF(ISNUMBER(S17),IF(S18&gt;S17,1.0,IF(S18=S17,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V18" s="15">
-        <f>IF(ISNUMBER(T18),IF(ISNUMBER(T17),IF(T18&gt;T17,1.0,IF(T18=T17,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T18),IF(ISNUMBER(T17),IF(T18&gt;T17,1.0,IF(T18=T17,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W18" s="21">
@@ -2493,11 +2493,11 @@
         <v/>
       </c>
       <c r="U19" s="14">
-        <f>IF(ISNUMBER(S19),IF(ISNUMBER(S20),IF(S19&gt;S20,1.0,IF(S19=S20,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S19),IF(ISNUMBER(S20),IF(S19&gt;S20,1.0,IF(S19=S20,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V19">
-        <f>IF(ISNUMBER(T19),IF(ISNUMBER(T20),IF(T19&gt;T20,1.0,IF(T19=T20,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T19),IF(ISNUMBER(T20),IF(T19&gt;T20,1.0,IF(T19=T20,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W19" s="14">
@@ -2588,11 +2588,11 @@
         <v/>
       </c>
       <c r="U20" s="21">
-        <f>IF(ISNUMBER(S20),IF(ISNUMBER(S19),IF(S20&gt;S19,1.0,IF(S20=S19,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S20),IF(ISNUMBER(S19),IF(S20&gt;S19,1.0,IF(S20=S19,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V20" s="15">
-        <f>IF(ISNUMBER(T20),IF(ISNUMBER(T19),IF(T20&gt;T19,1.0,IF(T20=T19,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T20),IF(ISNUMBER(T19),IF(T20&gt;T19,1.0,IF(T20=T19,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W20" s="21">
@@ -2685,11 +2685,11 @@
         <v/>
       </c>
       <c r="U21" s="14">
-        <f>IF(ISNUMBER(S21),IF(ISNUMBER(S22),IF(S21&gt;S22,1.0,IF(S21=S22,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S21),IF(ISNUMBER(S22),IF(S21&gt;S22,1.0,IF(S21=S22,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V21">
-        <f>IF(ISNUMBER(T21),IF(ISNUMBER(T22),IF(T21&gt;T22,1.0,IF(T21=T22,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T21),IF(ISNUMBER(T22),IF(T21&gt;T22,1.0,IF(T21=T22,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W21" s="14">
@@ -2780,11 +2780,11 @@
         <v/>
       </c>
       <c r="U22" s="21">
-        <f>IF(ISNUMBER(S22),IF(ISNUMBER(S21),IF(S22&gt;S21,1.0,IF(S22=S21,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S22),IF(ISNUMBER(S21),IF(S22&gt;S21,1.0,IF(S22=S21,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V22" s="15">
-        <f>IF(ISNUMBER(T22),IF(ISNUMBER(T21),IF(T22&gt;T21,1.0,IF(T22=T21,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T22),IF(ISNUMBER(T21),IF(T22&gt;T21,1.0,IF(T22=T21,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W22" s="21">
@@ -2877,11 +2877,11 @@
         <v/>
       </c>
       <c r="U23" s="14">
-        <f>IF(ISNUMBER(S23),IF(ISNUMBER(S24),IF(S23&gt;S24,1.0,IF(S23=S24,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S23),IF(ISNUMBER(S24),IF(S23&gt;S24,1.0,IF(S23=S24,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V23">
-        <f>IF(ISNUMBER(T23),IF(ISNUMBER(T24),IF(T23&gt;T24,1.0,IF(T23=T24,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T23),IF(ISNUMBER(T24),IF(T23&gt;T24,1.0,IF(T23=T24,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W23" s="14">
@@ -2972,11 +2972,11 @@
         <v/>
       </c>
       <c r="U24" s="21">
-        <f>IF(ISNUMBER(S24),IF(ISNUMBER(S23),IF(S24&gt;S23,1.0,IF(S24=S23,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S24),IF(ISNUMBER(S23),IF(S24&gt;S23,1.0,IF(S24=S23,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V24" s="15">
-        <f>IF(ISNUMBER(T24),IF(ISNUMBER(T23),IF(T24&gt;T23,1.0,IF(T24=T23,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T24),IF(ISNUMBER(T23),IF(T24&gt;T23,1.0,IF(T24=T23,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W24" s="21">
@@ -3069,11 +3069,11 @@
         <v/>
       </c>
       <c r="U25" s="14">
-        <f>IF(ISNUMBER(S25),IF(ISNUMBER(S26),IF(S25&gt;S26,1.0,IF(S25=S26,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S25),IF(ISNUMBER(S26),IF(S25&gt;S26,1.0,IF(S25=S26,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V25">
-        <f>IF(ISNUMBER(T25),IF(ISNUMBER(T26),IF(T25&gt;T26,1.0,IF(T25=T26,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T25),IF(ISNUMBER(T26),IF(T25&gt;T26,1.0,IF(T25=T26,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W25" s="14">
@@ -3164,11 +3164,11 @@
         <v/>
       </c>
       <c r="U26" s="21">
-        <f>IF(ISNUMBER(S26),IF(ISNUMBER(S25),IF(S26&gt;S25,1.0,IF(S26=S25,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S26),IF(ISNUMBER(S25),IF(S26&gt;S25,1.0,IF(S26=S25,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V26" s="15">
-        <f>IF(ISNUMBER(T26),IF(ISNUMBER(T25),IF(T26&gt;T25,1.0,IF(T26=T25,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T26),IF(ISNUMBER(T25),IF(T26&gt;T25,1.0,IF(T26=T25,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W26" s="21">
@@ -3261,11 +3261,11 @@
         <v/>
       </c>
       <c r="U27" s="14">
-        <f>IF(ISNUMBER(S27),IF(ISNUMBER(S28),IF(S27&gt;S28,1.0,IF(S27=S28,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S27),IF(ISNUMBER(S28),IF(S27&gt;S28,1.0,IF(S27=S28,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V27">
-        <f>IF(ISNUMBER(T27),IF(ISNUMBER(T28),IF(T27&gt;T28,1.0,IF(T27=T28,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T27),IF(ISNUMBER(T28),IF(T27&gt;T28,1.0,IF(T27=T28,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W27" s="14">
@@ -3356,11 +3356,11 @@
         <v/>
       </c>
       <c r="U28" s="21">
-        <f>IF(ISNUMBER(S28),IF(ISNUMBER(S27),IF(S28&gt;S27,1.0,IF(S28=S27,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S28),IF(ISNUMBER(S27),IF(S28&gt;S27,1.0,IF(S28=S27,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V28" s="15">
-        <f>IF(ISNUMBER(T28),IF(ISNUMBER(T27),IF(T28&gt;T27,1.0,IF(T28=T27,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T28),IF(ISNUMBER(T27),IF(T28&gt;T27,1.0,IF(T28=T27,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W28" s="21">
@@ -3453,11 +3453,11 @@
         <v/>
       </c>
       <c r="U29" s="14">
-        <f>IF(ISNUMBER(S29),IF(ISNUMBER(S30),IF(S29&gt;S30,1.0,IF(S29=S30,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S29),IF(ISNUMBER(S30),IF(S29&gt;S30,1.0,IF(S29=S30,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V29">
-        <f>IF(ISNUMBER(T29),IF(ISNUMBER(T30),IF(T29&gt;T30,1.0,IF(T29=T30,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T29),IF(ISNUMBER(T30),IF(T29&gt;T30,1.0,IF(T29=T30,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W29" s="14">
@@ -3548,11 +3548,11 @@
         <v/>
       </c>
       <c r="U30" s="21">
-        <f>IF(ISNUMBER(S30),IF(ISNUMBER(S29),IF(S30&gt;S29,1.0,IF(S30=S29,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S30),IF(ISNUMBER(S29),IF(S30&gt;S29,1.0,IF(S30=S29,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V30" s="15">
-        <f>IF(ISNUMBER(T30),IF(ISNUMBER(T29),IF(T30&gt;T29,1.0,IF(T30=T29,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T30),IF(ISNUMBER(T29),IF(T30&gt;T29,1.0,IF(T30=T29,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W30" s="21">
@@ -3645,11 +3645,11 @@
         <v/>
       </c>
       <c r="U31" s="14">
-        <f>IF(ISNUMBER(S31),IF(ISNUMBER(S32),IF(S31&gt;S32,1.0,IF(S31=S32,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S31),IF(ISNUMBER(S32),IF(S31&gt;S32,1.0,IF(S31=S32,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V31">
-        <f>IF(ISNUMBER(T31),IF(ISNUMBER(T32),IF(T31&gt;T32,1.0,IF(T31=T32,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T31),IF(ISNUMBER(T32),IF(T31&gt;T32,1.0,IF(T31=T32,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W31" s="14">
@@ -3740,11 +3740,11 @@
         <v/>
       </c>
       <c r="U32" s="21">
-        <f>IF(ISNUMBER(S32),IF(ISNUMBER(S31),IF(S32&gt;S31,1.0,IF(S32=S31,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S32),IF(ISNUMBER(S31),IF(S32&gt;S31,1.0,IF(S32=S31,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V32" s="15">
-        <f>IF(ISNUMBER(T32),IF(ISNUMBER(T31),IF(T32&gt;T31,1.0,IF(T32=T31,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T32),IF(ISNUMBER(T31),IF(T32&gt;T31,1.0,IF(T32=T31,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W32" s="21">
@@ -3837,11 +3837,11 @@
         <v/>
       </c>
       <c r="U33" s="14">
-        <f>IF(ISNUMBER(S33),IF(ISNUMBER(S34),IF(S33&gt;S34,1.0,IF(S33=S34,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S33),IF(ISNUMBER(S34),IF(S33&gt;S34,1.0,IF(S33=S34,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V33">
-        <f>IF(ISNUMBER(T33),IF(ISNUMBER(T34),IF(T33&gt;T34,1.0,IF(T33=T34,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T33),IF(ISNUMBER(T34),IF(T33&gt;T34,1.0,IF(T33=T34,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W33" s="14">
@@ -3932,11 +3932,11 @@
         <v/>
       </c>
       <c r="U34" s="21">
-        <f>IF(ISNUMBER(S34),IF(ISNUMBER(S33),IF(S34&gt;S33,1.0,IF(S34=S33,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S34),IF(ISNUMBER(S33),IF(S34&gt;S33,1.0,IF(S34=S33,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V34" s="15">
-        <f>IF(ISNUMBER(T34),IF(ISNUMBER(T33),IF(T34&gt;T33,1.0,IF(T34=T33,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T34),IF(ISNUMBER(T33),IF(T34&gt;T33,1.0,IF(T34=T33,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W34" s="21">
@@ -4029,11 +4029,11 @@
         <v/>
       </c>
       <c r="U35" s="14">
-        <f>IF(ISNUMBER(S35),IF(ISNUMBER(S36),IF(S35&gt;S36,1.0,IF(S35=S36,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S35),IF(ISNUMBER(S36),IF(S35&gt;S36,1.0,IF(S35=S36,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V35">
-        <f>IF(ISNUMBER(T35),IF(ISNUMBER(T36),IF(T35&gt;T36,1.0,IF(T35=T36,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T35),IF(ISNUMBER(T36),IF(T35&gt;T36,1.0,IF(T35=T36,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W35" s="14">
@@ -4124,11 +4124,11 @@
         <v/>
       </c>
       <c r="U36" s="21">
-        <f>IF(ISNUMBER(S36),IF(ISNUMBER(S35),IF(S36&gt;S35,1.0,IF(S36=S35,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S36),IF(ISNUMBER(S35),IF(S36&gt;S35,1.0,IF(S36=S35,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V36" s="15">
-        <f>IF(ISNUMBER(T36),IF(ISNUMBER(T35),IF(T36&gt;T35,1.0,IF(T36=T35,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T36),IF(ISNUMBER(T35),IF(T36&gt;T35,1.0,IF(T36=T35,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W36" s="21">
@@ -4221,11 +4221,11 @@
         <v/>
       </c>
       <c r="U37" s="14">
-        <f>IF(ISNUMBER(S37),IF(ISNUMBER(S38),IF(S37&gt;S38,1.0,IF(S37=S38,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S37),IF(ISNUMBER(S38),IF(S37&gt;S38,1.0,IF(S37=S38,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V37">
-        <f>IF(ISNUMBER(T37),IF(ISNUMBER(T38),IF(T37&gt;T38,1.0,IF(T37=T38,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T37),IF(ISNUMBER(T38),IF(T37&gt;T38,1.0,IF(T37=T38,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W37" s="14">
@@ -4316,11 +4316,11 @@
         <v/>
       </c>
       <c r="U38" s="21">
-        <f>IF(ISNUMBER(S38),IF(ISNUMBER(S37),IF(S38&gt;S37,1.0,IF(S38=S37,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(S38),IF(ISNUMBER(S37),IF(S38&gt;S37,1.0,IF(S38=S37,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="V38" s="15">
-        <f>IF(ISNUMBER(T38),IF(ISNUMBER(T37),IF(T38&gt;T37,1.0,IF(T38=T37,0.5,0.0)),""),"")</f>
+        <f>IF(ISNUMBER(T38),IF(ISNUMBER(T37),IF(T38&gt;T37,1.0,IF(T38=T37,0.5,0.0)),0.5),0.5)</f>
         <v/>
       </c>
       <c r="W38" s="21">

</xml_diff>